<commit_message>
docs(deliverables): supplement form replaces the removed medicine add row; 30-Oct sheet rebuilt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Design Deliverables 30-Oct-2026.xlsx
+++ b/Design Deliverables 30-Oct-2026.xlsx
@@ -3533,12 +3533,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Add to your record (medicine form)</t>
+          <t>Add to your record (supplement form)</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/record/add?kind=medicines</t>
+          <t>https://human-optimization-lab.vercel.app/app/record/add?kind=supplements</t>
         </is>
       </c>
     </row>

</xml_diff>